<commit_message>
Add secure SQU and Industry onboarding
</commit_message>
<xml_diff>
--- a/docs/examples/imports/exemple_initialisation_minimale_fyp_2028_2029.xlsx
+++ b/docs/examples/imports/exemple_initialisation_minimale_fyp_2028_2029.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="1" r:id="Rcd52141784534b00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRACKS" sheetId="2" r:id="R7304f61fcc52481f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STUDENTS" sheetId="3" r:id="Re6edbcc2f6aa492e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTORS" sheetId="4" r:id="R26d9a395cc9845e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROJECTS" sheetId="5" r:id="Re36d70f3d9f04dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEAM_MEMBERS" sheetId="6" r:id="Rcdecbd89ec324656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPERVISORS" sheetId="7" r:id="R1e6001d58c994712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVALUATOR_ASSIGNMENTS" sheetId="8" r:id="Ra0ecc45311664be4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASES" sheetId="9" r:id="Reb94f2f5575344bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCE_LISTS" sheetId="10" r:id="R5ae9721f23eb4148"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXAMPLES" sheetId="11" r:id="Red102af64ca54dc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTRUCTIONS" sheetId="1" r:id="Rfe6e8be3226e496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRACKS" sheetId="2" r:id="R16310d42c8714291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STUDENTS" sheetId="3" r:id="R70f46734607e4368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTORS" sheetId="4" r:id="Rbdaaa71eee324465"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROJECTS" sheetId="5" r:id="R0055c67f37c1420a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEAM_MEMBERS" sheetId="6" r:id="R36ae27ad84d34d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUPERVISORS" sheetId="7" r:id="Rbff3e07686f94d88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EVALUATOR_ASSIGNMENTS" sheetId="8" r:id="R1d906da7f3ce4f59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PHASES" sheetId="9" r:id="R97a1e20af8c247df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REFERENCE_LISTS" sheetId="10" r:id="R6ba86e4281324401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXAMPLES" sheetId="11" r:id="R898d3040ade84023"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1472,7 +1472,7 @@
         <x:v>ACTORS</x:v>
       </x:c>
       <x:c r="B16" s="65" t="str">
-        <x:v>Login accounts and evaluator profiles</x:v>
+        <x:v>SSO identities and invited Industry profiles</x:v>
       </x:c>
       <x:c r="C16" s="65" t="str">
         <x:v>Assignments</x:v>
@@ -1490,7 +1490,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="H16" s="66" t="str">
-        <x:v>New accounts require a temporary password</x:v>
+        <x:v>Internal: SQU SSO. Industry: expiry date and one-time invitation.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="38" customHeight="1">
@@ -1705,7 +1705,7 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="115" t="str">
-        <x:v>Minimal example: one PSE project and all three evaluator roles. All names and contacts are fictional. Import accounts use a temporary Demo@20xx password shown in ACTORS.</x:v>
+        <x:v>Minimal example: one PSE project and all three evaluator roles. All names and contacts are fictional. Internal actors use SQU SSO; the Industry Guest receives a one-time invitation link.</x:v>
       </x:c>
       <x:c r="B29" s="115"/>
       <x:c r="C29" s="115"/>
@@ -1820,7 +1820,7 @@
         <x:v>SUPERVISOR</x:v>
       </x:c>
       <x:c r="B3" s="93" t="str">
-        <x:v>INACTIVE</x:v>
+        <x:v>PENDING_INVITATION</x:v>
       </x:c>
       <x:c r="C3" s="93" t="str">
         <x:v>CSN</x:v>
@@ -1846,7 +1846,7 @@
         <x:v>FACULTY_EVALUATOR</x:v>
       </x:c>
       <x:c r="B4" s="93" t="str">
-        <x:v>SUSPENDED</x:v>
+        <x:v>INACTIVE</x:v>
       </x:c>
       <x:c r="C4" s="93" t="str">
         <x:v>CSP</x:v>
@@ -1867,7 +1867,9 @@
       <x:c r="A5" s="92" t="str">
         <x:v>INDUSTRY_REPRESENTATIVE</x:v>
       </x:c>
-      <x:c r="B5" s="93"/>
+      <x:c r="B5" s="93" t="str">
+        <x:v>SUSPENDED</x:v>
+      </x:c>
       <x:c r="C5" s="93" t="str">
         <x:v>PSE</x:v>
       </x:c>
@@ -1992,16 +1994,16 @@
         <x:v>ACTORS</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>SUP001 | Dr Sara Al Busaidi | sara@squ.edu.om | SUPERVISOR | Electrical Engineering | Power Systems | [blank] | +968... | ChangeMe@123 | ACTIVE</x:v>
+        <x:v>SUP001 | Dr Sara Al Busaidi | sara@squ.edu.om | SUPERVISOR | Electrical Engineering | Power Systems | [blank] | +968... | [blank] | ACTIVE</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
-        <x:v>IND001 | Ahmed Al Lawati | ahmed@industry.om | INDUSTRY_REPRESENTATIVE | [blank] | [blank] | Oman Energy | +968... | ChangeMe@123 | ACTIVE</x:v>
+        <x:v>IND001 | Ahmed Al Lawati | ahmed@industry.om | INDUSTRY_REPRESENTATIVE | [blank] | [blank] | Oman Energy | +968... | 2027-06-30 23:59 | PENDING_INVITATION</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
         <x:v>Accounts that can sign in</x:v>
       </x:c>
       <x:c r="E6" s="23" t="str">
-        <x:v>No STUDENT role; new account requires password</x:v>
+        <x:v>Internal email must be @squ.edu.om; Industry requires future accessExpiresAt and PENDING_INVITATION</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="64" customHeight="1">
@@ -5164,9 +5166,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bdbfb7841d6459f"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19f5cb48e9bb412c"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4508158c4e64863"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67721659bf184a2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9733,9 +9735,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac0c2dc43744f07"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65509403b7ec4679"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra696c62ccb084898"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R204fac2355ec4485"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9752,8 +9754,8 @@
     <x:col min="6" max="6" width="26" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="30" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="22" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="15" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -9782,7 +9784,7 @@
         <x:v>phone</x:v>
       </x:c>
       <x:c r="I1" s="73" t="str">
-        <x:v>temporaryPassword</x:v>
+        <x:v>accessExpiresAt</x:v>
       </x:c>
       <x:c r="J1" s="73" t="str">
         <x:v>status</x:v>
@@ -9811,9 +9813,7 @@
       <x:c r="H2" s="130" t="str">
         <x:v>+968 2400 2101</x:v>
       </x:c>
-      <x:c r="I2" s="130" t="str">
-        <x:v>Demo@2029</x:v>
-      </x:c>
+      <x:c r="I2" s="130"/>
       <x:c r="J2" s="131" t="str">
         <x:v>ACTIVE</x:v>
       </x:c>
@@ -9841,9 +9841,7 @@
       <x:c r="H3" s="132" t="str">
         <x:v>+968 2400 2201</x:v>
       </x:c>
-      <x:c r="I3" s="132" t="str">
-        <x:v>Demo@2029</x:v>
-      </x:c>
+      <x:c r="I3" s="132"/>
       <x:c r="J3" s="132" t="str">
         <x:v>ACTIVE</x:v>
       </x:c>
@@ -9872,10 +9870,10 @@
         <x:v>+968 9900 2301</x:v>
       </x:c>
       <x:c r="I4" s="132" t="str">
-        <x:v>Demo@2029</x:v>
+        <x:v>2029-06-30 23:59</x:v>
       </x:c>
       <x:c r="J4" s="132" t="str">
-        <x:v>ACTIVE</x:v>
+        <x:v>PENDING_INVITATION</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -15831,18 +15829,21 @@
       <x:c r="J500" s="74"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D2:D500">
       <x:formula1>'REFERENCE_LISTS'!$A$2:$A$6</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J500">
       <x:formula1>'REFERENCE_LISTS'!$B$2:$B$4</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="J2:J200">
+      <x:formula1>'REFERENCE_LISTS'!$B$2:$B$5</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re36a00109ca74e23"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b12cd12ebb1487a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0926678babdf476c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c9d03ffd9ff42c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20903,9 +20904,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc667a003c8704b39"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a18ccf1120549a9"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd90718c34974d18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a3c84779d334e89"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22932,9 +22933,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R253909adc5b84293"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3525d2ed4fb44987"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R789d0950b5ca40af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45e7061a767415b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -24957,9 +24958,9 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad778784d464775"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39b1ef72b46f4bcd"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40670dd4d81847dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R832a2f789021461f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -27516,9 +27517,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf25e16a8a8dd4dfe"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfea305d14da94563"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R800251b557684f90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R23627d9f0bbb43ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -31581,9 +31582,9 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c529c56c3e14aa5"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4637f2a68136441a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra839399fc0c24406"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1007ecad336e4756"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>